<commit_message>
style(ui): reubicacion topologica del selector de Sala Quirurgica justo despues de la captura de Hora en la seccion de programación
</commit_message>
<xml_diff>
--- a/Secuencia de consistencia.xlsx
+++ b/Secuencia de consistencia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\JVP\ANTIGRAVITY\BackCQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{508001FC-2F0C-4BDA-B43B-54030EB4C1FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6DA7F4E-BC32-4694-A15F-00AA08F41B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{45E6B47E-9D2D-4262-ADDC-B58272C922EC}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="35">
   <si>
     <t>Paciente (DNI / HC)</t>
   </si>
@@ -36,9 +36,6 @@
     <t>Tipo de Intervención</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
     <t>Tipo Operación</t>
   </si>
   <si>
@@ -105,12 +102,6 @@
     <t>T5</t>
   </si>
   <si>
-    <t>¿Puede Editar?</t>
-  </si>
-  <si>
-    <t>Coponentes</t>
-  </si>
-  <si>
     <t>Boton "Confirmar Cirugía"</t>
   </si>
   <si>
@@ -120,7 +111,25 @@
     <t>Boton "Ingreso a Quirofano"</t>
   </si>
   <si>
-    <t>Validacion de campo requerido (campos no vacios, no nulos)</t>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>Tiempo</t>
+  </si>
+  <si>
+    <t>Componentes</t>
+  </si>
+  <si>
+    <t>Boton "Salida Paciente"</t>
+  </si>
+  <si>
+    <t>T1 &lt; T2 &lt; T3 &lt; T3 &lt; T4 &lt; T5</t>
+  </si>
+  <si>
+    <t>Los campos OBLIGATORIOS estan marcados con "SI"</t>
+  </si>
+  <si>
+    <t>Los campos DESHABILITADOS estan marcados con "SI"</t>
   </si>
 </sst>
 </file>
@@ -142,7 +151,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -161,8 +170,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -170,20 +191,74 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -192,6 +267,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFCCFFFF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -500,269 +580,534 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98B7950D-B1E1-4331-8149-D6F32257AB69}">
-  <dimension ref="D2:I24"/>
+  <dimension ref="B2:M25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="24" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.42578125" style="2" customWidth="1"/>
-    <col min="8" max="9" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="4.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="24.85546875" style="1" customWidth="1"/>
+    <col min="6" max="7" width="24.85546875" customWidth="1"/>
+    <col min="8" max="8" width="2.7109375" customWidth="1"/>
+    <col min="9" max="13" width="22.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D2" t="s">
+    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C2" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="I2" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C3" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="I3" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="11" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="E3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" s="2" t="s">
+      <c r="I5" s="11" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
+      <c r="J5" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" s="2" t="s">
+      <c r="L5" s="11" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="5" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D5" s="1" t="s">
+      <c r="M5" s="11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D7" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D8" s="1" t="s">
+      <c r="C9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B10" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D9" s="1" t="s">
+      <c r="C10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B11" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D10" s="1" t="s">
+      <c r="C11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B12" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D11" s="1" t="s">
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-    </row>
-    <row r="12" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D12" s="1" t="s">
+      <c r="C13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B14" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D13" s="1" t="s">
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+    </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B15" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-    </row>
-    <row r="14" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D14" s="1" t="s">
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B16" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-    </row>
-    <row r="15" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D15" s="1" t="s">
+      <c r="C16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B17" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D16" s="1" t="s">
+      <c r="C17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D17" s="1" t="s">
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H17" s="2"/>
-    </row>
-    <row r="18" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D18" s="1" t="s">
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G18" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H18" s="2"/>
-    </row>
-    <row r="19" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D19" s="1" t="s">
+      <c r="C20" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B21" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D20" s="1" t="s">
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="5"/>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B22" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-    </row>
-    <row r="21" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D21" s="1" t="s">
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B23" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-    </row>
-    <row r="22" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D22" s="1" t="s">
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B24" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G22" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D23" s="1" t="s">
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B25" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G23" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D24" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H24" s="2"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="I2:M2"/>
+    <mergeCell ref="I3:M3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(sync): sincronizacion manual con repositorio a peticion del usuario
</commit_message>
<xml_diff>
--- a/Secuencia de consistencia.xlsx
+++ b/Secuencia de consistencia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\JVP\ANTIGRAVITY\BackCQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6DA7F4E-BC32-4694-A15F-00AA08F41B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB27467-DE82-4088-A35B-31DA35B03503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{45E6B47E-9D2D-4262-ADDC-B58272C922EC}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="35">
   <si>
     <t>Paciente (DNI / HC)</t>
   </si>
@@ -714,7 +714,9 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
+      <c r="M6" s="5" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
@@ -735,7 +737,9 @@
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
+      <c r="M7" s="5" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
@@ -802,7 +806,9 @@
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
+      <c r="M10" s="5" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
@@ -825,7 +831,9 @@
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
       <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
+      <c r="M11" s="5" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
@@ -863,7 +871,9 @@
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
+      <c r="M13" s="5" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
@@ -916,7 +926,9 @@
       <c r="J16" s="5"/>
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
+      <c r="M16" s="5" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
@@ -939,7 +951,9 @@
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
+      <c r="M17" s="5" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
@@ -981,7 +995,9 @@
       <c r="J19" s="5"/>
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
+      <c r="M19" s="5" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">

</xml_diff>